<commit_message>
corrigido erro de CPF/CNPJ e integração de CEP automático
</commit_message>
<xml_diff>
--- a/empresas.xlsx
+++ b/empresas.xlsx
@@ -512,10 +512,8 @@
           <t>Avenida Jose Faria da Rocha</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>5970</t>
-        </is>
+      <c r="J2" t="n">
+        <v>5970</v>
       </c>
     </row>
     <row r="3">
@@ -562,10 +560,8 @@
           <t>Rua Curitiba</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>327</t>
-        </is>
+      <c r="J3" t="n">
+        <v>327</v>
       </c>
     </row>
     <row r="4">

</xml_diff>